<commit_message>
DetectCapital - String Problem
</commit_message>
<xml_diff>
--- a/DSA-TrackerSheet/RahulTakale-LeetcodeTrackerSheet.xlsx
+++ b/DSA-TrackerSheet/RahulTakale-LeetcodeTrackerSheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Leetcode-RahulTakale\DSA-TrackerSheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3962B0-D703-4551-AE8E-F3065D8B683F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{124C64ED-C4BD-4F42-8010-8B878CB0EB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3289,6 +3289,12 @@
     <xf numFmtId="9" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -3299,12 +3305,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3912,28 +3912,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.35" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="10" t="s">
         <v>1043</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="14"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="10"/>
     </row>
     <row r="3" spans="1:8" ht="15.6">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="12" t="s">
         <v>1028</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="4" t="s">
@@ -5423,16 +5423,16 @@
       </c>
     </row>
     <row r="72" spans="1:8" ht="15.6">
-      <c r="A72" s="10" t="s">
+      <c r="A72" s="12" t="s">
         <v>1030</v>
       </c>
-      <c r="B72" s="10"/>
-      <c r="C72" s="10"/>
-      <c r="D72" s="10"/>
-      <c r="E72" s="10"/>
-      <c r="F72" s="10"/>
-      <c r="G72" s="10"/>
-      <c r="H72" s="10"/>
+      <c r="B72" s="12"/>
+      <c r="C72" s="12"/>
+      <c r="D72" s="12"/>
+      <c r="E72" s="12"/>
+      <c r="F72" s="12"/>
+      <c r="G72" s="12"/>
+      <c r="H72" s="12"/>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" s="4" t="s">
@@ -6601,16 +6601,16 @@
       </c>
     </row>
     <row r="126" spans="1:8" ht="15.6">
-      <c r="A126" s="10" t="s">
+      <c r="A126" s="12" t="s">
         <v>1031</v>
       </c>
-      <c r="B126" s="10"/>
-      <c r="C126" s="10"/>
-      <c r="D126" s="10"/>
-      <c r="E126" s="10"/>
-      <c r="F126" s="10"/>
-      <c r="G126" s="10"/>
-      <c r="H126" s="10"/>
+      <c r="B126" s="12"/>
+      <c r="C126" s="12"/>
+      <c r="D126" s="12"/>
+      <c r="E126" s="12"/>
+      <c r="F126" s="12"/>
+      <c r="G126" s="12"/>
+      <c r="H126" s="12"/>
     </row>
     <row r="127" spans="1:8">
       <c r="A127" s="4" t="s">
@@ -7305,16 +7305,16 @@
       </c>
     </row>
     <row r="160" spans="1:8" ht="15.6">
-      <c r="A160" s="10" t="s">
+      <c r="A160" s="12" t="s">
         <v>1032</v>
       </c>
-      <c r="B160" s="10"/>
-      <c r="C160" s="10"/>
-      <c r="D160" s="10"/>
-      <c r="E160" s="10"/>
-      <c r="F160" s="10"/>
-      <c r="G160" s="10"/>
-      <c r="H160" s="10"/>
+      <c r="B160" s="12"/>
+      <c r="C160" s="12"/>
+      <c r="D160" s="12"/>
+      <c r="E160" s="12"/>
+      <c r="F160" s="12"/>
+      <c r="G160" s="12"/>
+      <c r="H160" s="12"/>
     </row>
     <row r="161" spans="1:8">
       <c r="A161" s="4" t="s">
@@ -8144,16 +8144,16 @@
       </c>
     </row>
     <row r="199" spans="1:8" ht="15.6">
-      <c r="A199" s="10" t="s">
+      <c r="A199" s="12" t="s">
         <v>1033</v>
       </c>
-      <c r="B199" s="10"/>
-      <c r="C199" s="10"/>
-      <c r="D199" s="10"/>
-      <c r="E199" s="10"/>
-      <c r="F199" s="10"/>
-      <c r="G199" s="10"/>
-      <c r="H199" s="10"/>
+      <c r="B199" s="12"/>
+      <c r="C199" s="12"/>
+      <c r="D199" s="12"/>
+      <c r="E199" s="12"/>
+      <c r="F199" s="12"/>
+      <c r="G199" s="12"/>
+      <c r="H199" s="12"/>
     </row>
     <row r="200" spans="1:8">
       <c r="A200" s="4" t="s">
@@ -8981,16 +8981,16 @@
       <c r="G235" s="2"/>
     </row>
     <row r="238" spans="1:8" ht="15.6">
-      <c r="A238" s="10" t="s">
+      <c r="A238" s="12" t="s">
         <v>1034</v>
       </c>
-      <c r="B238" s="10"/>
-      <c r="C238" s="10"/>
-      <c r="D238" s="10"/>
-      <c r="E238" s="10"/>
-      <c r="F238" s="10"/>
-      <c r="G238" s="10"/>
-      <c r="H238" s="10"/>
+      <c r="B238" s="12"/>
+      <c r="C238" s="12"/>
+      <c r="D238" s="12"/>
+      <c r="E238" s="12"/>
+      <c r="F238" s="12"/>
+      <c r="G238" s="12"/>
+      <c r="H238" s="12"/>
     </row>
     <row r="239" spans="1:8">
       <c r="A239" s="4" t="s">
@@ -10054,16 +10054,16 @@
       </c>
     </row>
     <row r="287" spans="1:8" ht="15.6">
-      <c r="A287" s="10" t="s">
+      <c r="A287" s="12" t="s">
         <v>1035</v>
       </c>
-      <c r="B287" s="10"/>
-      <c r="C287" s="10"/>
-      <c r="D287" s="10"/>
-      <c r="E287" s="10"/>
-      <c r="F287" s="10"/>
-      <c r="G287" s="10"/>
-      <c r="H287" s="10"/>
+      <c r="B287" s="12"/>
+      <c r="C287" s="12"/>
+      <c r="D287" s="12"/>
+      <c r="E287" s="12"/>
+      <c r="F287" s="12"/>
+      <c r="G287" s="12"/>
+      <c r="H287" s="12"/>
     </row>
     <row r="288" spans="1:8">
       <c r="A288" s="4" t="s">
@@ -11127,16 +11127,16 @@
       </c>
     </row>
     <row r="336" spans="1:8" ht="15.6">
-      <c r="A336" s="10" t="s">
+      <c r="A336" s="12" t="s">
         <v>1036</v>
       </c>
-      <c r="B336" s="10"/>
-      <c r="C336" s="10"/>
-      <c r="D336" s="10"/>
-      <c r="E336" s="10"/>
-      <c r="F336" s="10"/>
-      <c r="G336" s="10"/>
-      <c r="H336" s="10"/>
+      <c r="B336" s="12"/>
+      <c r="C336" s="12"/>
+      <c r="D336" s="12"/>
+      <c r="E336" s="12"/>
+      <c r="F336" s="12"/>
+      <c r="G336" s="12"/>
+      <c r="H336" s="12"/>
     </row>
     <row r="337" spans="1:8">
       <c r="A337" s="4" t="s">
@@ -12537,16 +12537,16 @@
       </c>
     </row>
     <row r="400" spans="1:8" ht="15.6">
-      <c r="A400" s="10" t="s">
+      <c r="A400" s="12" t="s">
         <v>1037</v>
       </c>
-      <c r="B400" s="10"/>
-      <c r="C400" s="10"/>
-      <c r="D400" s="10"/>
-      <c r="E400" s="10"/>
-      <c r="F400" s="10"/>
-      <c r="G400" s="10"/>
-      <c r="H400" s="10"/>
+      <c r="B400" s="12"/>
+      <c r="C400" s="12"/>
+      <c r="D400" s="12"/>
+      <c r="E400" s="12"/>
+      <c r="F400" s="12"/>
+      <c r="G400" s="12"/>
+      <c r="H400" s="12"/>
     </row>
     <row r="401" spans="1:8">
       <c r="A401" s="4" t="s">
@@ -13265,16 +13265,16 @@
       </c>
     </row>
     <row r="434" spans="1:8" ht="15.6">
-      <c r="A434" s="10" t="s">
+      <c r="A434" s="12" t="s">
         <v>1038</v>
       </c>
-      <c r="B434" s="10"/>
-      <c r="C434" s="10"/>
-      <c r="D434" s="10"/>
-      <c r="E434" s="10"/>
-      <c r="F434" s="10"/>
-      <c r="G434" s="10"/>
-      <c r="H434" s="10"/>
+      <c r="B434" s="12"/>
+      <c r="C434" s="12"/>
+      <c r="D434" s="12"/>
+      <c r="E434" s="12"/>
+      <c r="F434" s="12"/>
+      <c r="G434" s="12"/>
+      <c r="H434" s="12"/>
     </row>
     <row r="435" spans="1:8">
       <c r="A435" s="4" t="s">
@@ -13876,16 +13876,16 @@
       </c>
     </row>
     <row r="463" spans="1:8" ht="15.6">
-      <c r="A463" s="10" t="s">
+      <c r="A463" s="12" t="s">
         <v>1039</v>
       </c>
-      <c r="B463" s="10"/>
-      <c r="C463" s="10"/>
-      <c r="D463" s="10"/>
-      <c r="E463" s="10"/>
-      <c r="F463" s="10"/>
-      <c r="G463" s="10"/>
-      <c r="H463" s="10"/>
+      <c r="B463" s="12"/>
+      <c r="C463" s="12"/>
+      <c r="D463" s="12"/>
+      <c r="E463" s="12"/>
+      <c r="F463" s="12"/>
+      <c r="G463" s="12"/>
+      <c r="H463" s="12"/>
     </row>
     <row r="464" spans="1:8">
       <c r="A464" s="4" t="s">
@@ -14150,16 +14150,16 @@
       <c r="G476" s="2"/>
     </row>
     <row r="477" spans="1:8" ht="15.6">
-      <c r="A477" s="10" t="s">
+      <c r="A477" s="12" t="s">
         <v>1040</v>
       </c>
-      <c r="B477" s="10"/>
-      <c r="C477" s="10"/>
-      <c r="D477" s="10"/>
-      <c r="E477" s="10"/>
-      <c r="F477" s="10"/>
-      <c r="G477" s="11"/>
-      <c r="H477" s="10"/>
+      <c r="B477" s="12"/>
+      <c r="C477" s="12"/>
+      <c r="D477" s="12"/>
+      <c r="E477" s="12"/>
+      <c r="F477" s="12"/>
+      <c r="G477" s="13"/>
+      <c r="H477" s="12"/>
     </row>
     <row r="478" spans="1:8">
       <c r="A478" s="4" t="s">
@@ -14717,28 +14717,28 @@
       </c>
     </row>
     <row r="502" spans="1:8" ht="15.6">
-      <c r="A502" s="12">
+      <c r="A502" s="14">
         <v>454</v>
       </c>
-      <c r="B502" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="C502" s="13">
+      <c r="B502" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C502" s="15">
         <v>357</v>
       </c>
-      <c r="D502" s="13" t="s">
+      <c r="D502" s="15" t="s">
         <v>934</v>
       </c>
-      <c r="E502" s="13" t="s">
+      <c r="E502" s="15" t="s">
         <v>935</v>
       </c>
-      <c r="F502" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="G502" s="13">
+      <c r="F502" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="G502" s="15">
         <v>46438</v>
       </c>
-      <c r="H502" s="13"/>
+      <c r="H502" s="15"/>
     </row>
     <row r="503" spans="1:8">
       <c r="A503" s="3">
@@ -14771,16 +14771,16 @@
       <c r="G505" s="2"/>
     </row>
     <row r="506" spans="1:8" ht="15.6">
-      <c r="A506" s="10" t="s">
+      <c r="A506" s="12" t="s">
         <v>1041</v>
       </c>
-      <c r="B506" s="10"/>
-      <c r="C506" s="10"/>
-      <c r="D506" s="10"/>
-      <c r="E506" s="10"/>
-      <c r="F506" s="10"/>
-      <c r="G506" s="11"/>
-      <c r="H506" s="10"/>
+      <c r="B506" s="12"/>
+      <c r="C506" s="12"/>
+      <c r="D506" s="12"/>
+      <c r="E506" s="12"/>
+      <c r="F506" s="12"/>
+      <c r="G506" s="13"/>
+      <c r="H506" s="12"/>
     </row>
     <row r="507" spans="1:8">
       <c r="A507" s="4" t="s">
@@ -15108,28 +15108,28 @@
       </c>
     </row>
     <row r="521" spans="1:8" ht="15.6">
-      <c r="A521" s="12">
+      <c r="A521" s="14">
         <v>469</v>
       </c>
-      <c r="B521" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="C521" s="13">
+      <c r="B521" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C521" s="15">
         <v>1268</v>
       </c>
-      <c r="D521" s="13" t="s">
+      <c r="D521" s="15" t="s">
         <v>964</v>
       </c>
-      <c r="E521" s="13" t="s">
+      <c r="E521" s="15" t="s">
         <v>965</v>
       </c>
-      <c r="F521" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="G521" s="13">
+      <c r="F521" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="G521" s="15">
         <v>46443</v>
       </c>
-      <c r="H521" s="13"/>
+      <c r="H521" s="15"/>
     </row>
     <row r="522" spans="1:8">
       <c r="A522" s="3">
@@ -15162,16 +15162,16 @@
       <c r="G524" s="2"/>
     </row>
     <row r="525" spans="1:8" ht="15.6">
-      <c r="A525" s="10" t="s">
+      <c r="A525" s="12" t="s">
         <v>1042</v>
       </c>
-      <c r="B525" s="10"/>
-      <c r="C525" s="10"/>
-      <c r="D525" s="10"/>
-      <c r="E525" s="10"/>
-      <c r="F525" s="10"/>
-      <c r="G525" s="11"/>
-      <c r="H525" s="10"/>
+      <c r="B525" s="12"/>
+      <c r="C525" s="12"/>
+      <c r="D525" s="12"/>
+      <c r="E525" s="12"/>
+      <c r="F525" s="12"/>
+      <c r="G525" s="13"/>
+      <c r="H525" s="12"/>
     </row>
     <row r="526" spans="1:8">
       <c r="A526" s="4" t="s">
@@ -15885,16 +15885,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A72:H72"/>
-    <mergeCell ref="A126:H126"/>
-    <mergeCell ref="A160:H160"/>
-    <mergeCell ref="A199:H199"/>
-    <mergeCell ref="A238:H238"/>
-    <mergeCell ref="A287:H287"/>
-    <mergeCell ref="A336:H336"/>
-    <mergeCell ref="A400:H400"/>
     <mergeCell ref="A525:H525"/>
     <mergeCell ref="A434:H434"/>
     <mergeCell ref="A463:H463"/>
@@ -15902,6 +15892,16 @@
     <mergeCell ref="A521:H521"/>
     <mergeCell ref="A477:H477"/>
     <mergeCell ref="A506:H506"/>
+    <mergeCell ref="A199:H199"/>
+    <mergeCell ref="A238:H238"/>
+    <mergeCell ref="A287:H287"/>
+    <mergeCell ref="A336:H336"/>
+    <mergeCell ref="A400:H400"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A72:H72"/>
+    <mergeCell ref="A126:H126"/>
+    <mergeCell ref="A160:H160"/>
   </mergeCells>
   <conditionalFormatting sqref="F3:F555">
     <cfRule type="expression" dxfId="1" priority="1">

</xml_diff>